<commit_message>
new all data cleared
</commit_message>
<xml_diff>
--- a/pincodes.xlsx
+++ b/pincodes.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="14">
   <si>
     <t>pincode</t>
   </si>
@@ -35,12 +35,18 @@
     <t>city</t>
   </si>
   <si>
+    <t>state</t>
+  </si>
+  <si>
     <t>380001</t>
   </si>
   <si>
     <t>Ahmedabad</t>
   </si>
   <si>
+    <t>Gujarat</t>
+  </si>
+  <si>
     <t>380009</t>
   </si>
   <si>
@@ -60,6 +66,9 @@
   </si>
   <si>
     <t>Pune</t>
+  </si>
+  <si>
+    <t>Maharashtra</t>
   </si>
 </sst>
 </file>
@@ -1046,98 +1055,131 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="1"/>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="2"/>
   <cols>
     <col min="2" max="2" width="11.59375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
-        <v>3</v>
+      <c r="C3" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:3">
       <c r="A9">
         <v>380022</v>
       </c>
       <c r="B9" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:3">
       <c r="A10">
         <v>380025</v>
       </c>
       <c r="B10" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:3">
       <c r="A11">
         <v>412105</v>
       </c>
       <c r="B11" t="s">
-        <v>10</v>
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>